<commit_message>
remove old documentation files and add new ones
</commit_message>
<xml_diff>
--- a/data/raw/Archive.xlsx
+++ b/data/raw/Archive.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10817"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noemivillars-amberg/Documents/daschland-scripts/data/spreadsheets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noemivillars-amberg/Documents/Customer_Projects/daschland-scripts/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61A0B49B-E411-634E-8DD8-DC30D6B73402}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6648AAA6-0E7A-7342-A380-E110789E0805}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="620" windowWidth="63440" windowHeight="14140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3320" yWindow="600" windowWidth="63440" windowHeight="18640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="18">
   <si>
     <t>ID</t>
   </si>
@@ -58,20 +58,29 @@
     <t>CC BY 4.0</t>
   </si>
   <si>
-    <t>https://app.rdu-08.dasch.swiss/resource/0854/QAJPzaUuQ_qWjn1aRbVxUQ</t>
-  </si>
-  <si>
     <t>Daniela Subotic, Noémi Villars-Amberg</t>
   </si>
   <si>
     <t>Authorship Resource</t>
+  </si>
+  <si>
+    <t>AR_002</t>
+  </si>
+  <si>
+    <t>Documentation_Documents.zip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Archive of the files used to create the project documentation. </t>
+  </si>
+  <si>
+    <t>Noémi Villars-Amberg</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -84,6 +93,12 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -423,7 +438,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.5" bestFit="1" customWidth="1"/>
@@ -458,7 +473,7 @@
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -477,17 +492,38 @@
       <c r="E2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>12</v>
       </c>
-      <c r="G2" t="s">
-        <v>13</v>
-      </c>
       <c r="H2" t="s">
-        <v>13</v>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Naming and descriptions update
</commit_message>
<xml_diff>
--- a/data/raw/Archive.xlsx
+++ b/data/raw/Archive.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noemivillars-amberg/Documents/Customer_Projects/daschland-scripts/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6648AAA6-0E7A-7342-A380-E110789E0805}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06BFC764-881D-1149-95E2-D4C0CE918EA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3320" yWindow="600" windowWidth="63440" windowHeight="18640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="35500" yWindow="3660" windowWidth="27960" windowHeight="18640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -67,13 +67,13 @@
     <t>AR_002</t>
   </si>
   <si>
-    <t>Documentation_Documents.zip</t>
-  </si>
-  <si>
     <t xml:space="preserve">Archive of the files used to create the project documentation. </t>
   </si>
   <si>
     <t>Noémi Villars-Amberg</t>
+  </si>
+  <si>
+    <t>Documentation_Source.zip</t>
   </si>
 </sst>
 </file>
@@ -504,10 +504,10 @@
         <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D3" t="s">
         <v>10</v>
@@ -516,10 +516,10 @@
         <v>11</v>
       </c>
       <c r="G3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
remove old documentation files and add new ones (#123)
</commit_message>
<xml_diff>
--- a/data/raw/Archive.xlsx
+++ b/data/raw/Archive.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10817"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noemivillars-amberg/Documents/daschland-scripts/data/spreadsheets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noemivillars-amberg/Documents/Customer_Projects/daschland-scripts/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61A0B49B-E411-634E-8DD8-DC30D6B73402}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06BFC764-881D-1149-95E2-D4C0CE918EA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="620" windowWidth="63440" windowHeight="14140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="35500" yWindow="3660" windowWidth="27960" windowHeight="18640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="18">
   <si>
     <t>ID</t>
   </si>
@@ -58,20 +58,29 @@
     <t>CC BY 4.0</t>
   </si>
   <si>
-    <t>https://app.rdu-08.dasch.swiss/resource/0854/QAJPzaUuQ_qWjn1aRbVxUQ</t>
-  </si>
-  <si>
     <t>Daniela Subotic, Noémi Villars-Amberg</t>
   </si>
   <si>
     <t>Authorship Resource</t>
+  </si>
+  <si>
+    <t>AR_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Archive of the files used to create the project documentation. </t>
+  </si>
+  <si>
+    <t>Noémi Villars-Amberg</t>
+  </si>
+  <si>
+    <t>Documentation_Source.zip</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -84,6 +93,12 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -423,7 +438,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.5" bestFit="1" customWidth="1"/>
@@ -458,7 +473,7 @@
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -477,17 +492,38 @@
       <c r="E2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>12</v>
       </c>
-      <c r="G2" t="s">
-        <v>13</v>
-      </c>
       <c r="H2" t="s">
-        <v>13</v>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H3" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>